<commit_message>
Restore merged cells in example workbook
</commit_message>
<xml_diff>
--- a/app/base/250927_오펄스_작성예제.xlsx
+++ b/app/base/250927_오펄스_작성예제.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="채널시트 작성 예제" sheetId="1" r:id="R2a8d48292c8f4b21"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="채널시트 작성 예제" sheetId="1" r:id="R71233516ea8a4f82"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1427,6 +1427,38 @@
       <x:c r="L41" s="13"/>
     </x:row>
   </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="C10:C11"/>
+    <x:mergeCell ref="C12:C13"/>
+    <x:mergeCell ref="C14:C15"/>
+    <x:mergeCell ref="C16:C17"/>
+    <x:mergeCell ref="D10:D11"/>
+    <x:mergeCell ref="D12:D13"/>
+    <x:mergeCell ref="D14:D15"/>
+    <x:mergeCell ref="D16:D17"/>
+    <x:mergeCell ref="I10:I11"/>
+    <x:mergeCell ref="I12:I13"/>
+    <x:mergeCell ref="I14:I15"/>
+    <x:mergeCell ref="I18:I21"/>
+    <x:mergeCell ref="I2:I3"/>
+    <x:mergeCell ref="I4:I5"/>
+    <x:mergeCell ref="I6:I7"/>
+    <x:mergeCell ref="I8:I9"/>
+    <x:mergeCell ref="J10:J11"/>
+    <x:mergeCell ref="J12:J13"/>
+    <x:mergeCell ref="J14:J15"/>
+    <x:mergeCell ref="J8:J9"/>
+    <x:mergeCell ref="K10:K11"/>
+    <x:mergeCell ref="K12:K13"/>
+    <x:mergeCell ref="K14:K15"/>
+    <x:mergeCell ref="K6:K7"/>
+    <x:mergeCell ref="K8:K9"/>
+    <x:mergeCell ref="L22:L23"/>
+    <x:mergeCell ref="L2:L3"/>
+    <x:mergeCell ref="L4:L5"/>
+    <x:mergeCell ref="L6:L7"/>
+    <x:mergeCell ref="L8:L9"/>
+  </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
 </file>
</xml_diff>